<commit_message>
Fix duplicate merge and customer purchase import
</commit_message>
<xml_diff>
--- a/public/mau_nhap_mua_tu_khach.xlsx
+++ b/public/mau_nhap_mua_tu_khach.xlsx
@@ -64,11 +64,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -124,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
-        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
-        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
-        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
+        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -159,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
-        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
-        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
-        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
+        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -402,11 +401,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:R2"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="16.875"/>
+    <col min="1" max="1" width="20.625" customWidth="1"/>
     <col min="2" max="2" customWidth="1" width="17.75"/>
     <col min="3" max="3" customWidth="1" width="21.625"/>
     <col min="5" max="5" customWidth="1" width="15.375"/>
-    <col min="6" max="6" width="24.625" customWidth="1"/>
+    <col min="6" max="6" customWidth="1" width="24.625"/>
     <col min="7" max="7" customWidth="1" width="17.25"/>
     <col min="8" max="8" customWidth="1" width="18.125"/>
     <col min="14" max="14" customWidth="1" width="13.125"/>
@@ -417,7 +416,7 @@
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
       <c r="A1" t="str">
-        <v>Ngày mua</v>
+        <v>Ngày mua (YYYY-MM-DD)</v>
       </c>
       <c r="B1" t="str">
         <v>Tên khách hàng</v>
@@ -472,8 +471,8 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3">
-        <v>46153</v>
+      <c r="A2" s="1" t="str">
+        <v>2026-05-25</v>
       </c>
       <c r="B2" t="str">
         <v>Vũ Thị Hà</v>

</xml_diff>